<commit_message>
20260311 update report Details
</commit_message>
<xml_diff>
--- a/reports.xlsx
+++ b/reports.xlsx
@@ -1,19 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IOtel\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{745FBCCF-4DCB-4880-A710-4DBE5CC06DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3087E1C1-5620-4352-9E20-971223EA9F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="17280" windowHeight="10500" xr2:uid="{4A38C952-6B38-47C9-B6BD-60FF9586BBD2}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" firstSheet="1" activeTab="1" xr2:uid="{4A38C952-6B38-47C9-B6BD-60FF9586BBD2}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Reports" sheetId="1" r:id="rId1"/>
+    <sheet name="Schedules" sheetId="2" r:id="rId2"/>
+    <sheet name="Functions" sheetId="3" r:id="rId3"/>
+    <sheet name="Tags" sheetId="4" r:id="rId4"/>
+    <sheet name="Changes" sheetId="5" r:id="rId5"/>
+    <sheet name="SQL Statements" sheetId="6" r:id="rId6"/>
+    <sheet name="Tables" sheetId="7" r:id="rId7"/>
+    <sheet name="Publications" sheetId="8" r:id="rId8"/>
+    <sheet name="Linked Reports" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,30 +43,147 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
-  <si>
-    <t>begin</t>
-  </si>
-  <si>
-    <t>lees filter</t>
-  </si>
-  <si>
-    <t>filtype = leeg</t>
-  </si>
-  <si>
-    <t>filtype='reportType'</t>
-  </si>
-  <si>
-    <t>filtype = nie leeg</t>
-  </si>
-  <si>
-    <t>nie begin</t>
-  </si>
-  <si>
-    <t>fildet=filter.reportType</t>
-  </si>
-  <si>
-    <t>doen bywerking van filter tov filtype</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="47">
+  <si>
+    <t>Crystal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required </t>
+  </si>
+  <si>
+    <t>Report</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Path</t>
+  </si>
+  <si>
+    <t>Components</t>
+  </si>
+  <si>
+    <t>Schedules</t>
+  </si>
+  <si>
+    <t>Functions</t>
+  </si>
+  <si>
+    <t>Tags</t>
+  </si>
+  <si>
+    <t>Changes</t>
+  </si>
+  <si>
+    <t>SQL statement</t>
+  </si>
+  <si>
+    <t>Tables</t>
+  </si>
+  <si>
+    <t>Add report</t>
+  </si>
+  <si>
+    <t>Edit Report</t>
+  </si>
+  <si>
+    <t>Remove Report</t>
+  </si>
+  <si>
+    <t>Select ion</t>
+  </si>
+  <si>
+    <t>Selection</t>
+  </si>
+  <si>
+    <t>Add</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add </t>
+  </si>
+  <si>
+    <t>View DB</t>
+  </si>
+  <si>
+    <t>Link Table</t>
+  </si>
+  <si>
+    <t>PHP</t>
+  </si>
+  <si>
+    <t>Recipients</t>
+  </si>
+  <si>
+    <t>Publications</t>
+  </si>
+  <si>
+    <t>Publication</t>
+  </si>
+  <si>
+    <t>Linked Reports</t>
+  </si>
+  <si>
+    <t>Filter</t>
+  </si>
+  <si>
+    <t>sh</t>
+  </si>
+  <si>
+    <t>View</t>
+  </si>
+  <si>
+    <t>Edit</t>
+  </si>
+  <si>
+    <t>Remove</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Report selection</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>DB selection</t>
+  </si>
+  <si>
+    <t>Link Tables</t>
+  </si>
+  <si>
+    <t>DB Add</t>
+  </si>
+  <si>
+    <t>Link  Table</t>
+  </si>
+  <si>
+    <t>Table Selection</t>
+  </si>
+  <si>
+    <t>Crystal / PHP / Recipients</t>
+  </si>
+  <si>
+    <t>Se;lection</t>
+  </si>
+  <si>
+    <t>Crystal / Recipients</t>
+  </si>
+  <si>
+    <t>Show report Group</t>
+  </si>
+  <si>
+    <t>View Ricipients</t>
+  </si>
+  <si>
+    <t>View Report Schedule</t>
+  </si>
+  <si>
+    <t>View Publication  Schedule</t>
   </si>
 </sst>
 </file>
@@ -74,12 +199,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -94,10 +225,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="5"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -418,56 +567,869 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C6B047-5BD0-4FE0-9344-E232D0E4E58E}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultColWidth="12.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
         <v>7</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="3" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="2" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85833828-42CF-4E9A-8919-B3F15621B530}">
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C8" s="7" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C9" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C10" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C11" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EFCA283-128B-472C-881B-44B4853A4854}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{485339A9-4BE2-45AB-8FCB-653A83302CB3}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3"/>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3"/>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D83B7FB6-87DE-4BE7-B4DF-F791D9A03C62}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8204F7E-C86F-4DDB-AB30-05192EA3866B}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{789D6D66-3E83-4E10-B02B-B18567320797}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F93FCF0B-DF71-4561-B3D8-C995E16F98A3}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ECFC2A7-8C30-4C6E-9B70-4D34865ED7BC}">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Changed Schedules and Functions Edit and Add
</commit_message>
<xml_diff>
--- a/reports.xlsx
+++ b/reports.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IOtel\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3087E1C1-5620-4352-9E20-971223EA9F00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F0062CD-9AE9-4236-9CB3-12C345F506E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" firstSheet="1" activeTab="1" xr2:uid="{4A38C952-6B38-47C9-B6BD-60FF9586BBD2}"/>
+    <workbookView xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="10500" activeTab="1" xr2:uid="{4A38C952-6B38-47C9-B6BD-60FF9586BBD2}"/>
   </bookViews>
   <sheets>
     <sheet name="Reports" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="49">
   <si>
     <t>Crystal</t>
   </si>
@@ -168,9 +168,6 @@
     <t>Crystal / PHP / Recipients</t>
   </si>
   <si>
-    <t>Se;lection</t>
-  </si>
-  <si>
     <t>Crystal / Recipients</t>
   </si>
   <si>
@@ -184,6 +181,15 @@
   </si>
   <si>
     <t>View Publication  Schedule</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>runTime</t>
+  </si>
+  <si>
+    <t>Dest Detail</t>
   </si>
 </sst>
 </file>
@@ -199,7 +205,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -209,6 +215,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -225,7 +237,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
@@ -243,10 +255,29 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" indent="5"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -567,7 +598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C6B047-5BD0-4FE0-9344-E232D0E4E58E}">
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultColWidth="12.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
@@ -591,87 +622,87 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="7" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="6" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="6" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="6" t="s">
         <v>5</v>
       </c>
     </row>
@@ -693,53 +724,44 @@
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="6" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="3" t="s">
+      <c r="A9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="C9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" s="3" t="s">
+      <c r="D9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="E9" s="8" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="3" t="s">
+      <c r="A10" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" s="8" t="s">
         <v>19</v>
       </c>
     </row>
@@ -747,68 +769,41 @@
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B11" s="2" t="s">
-        <v>9</v>
-      </c>
       <c r="C11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>10</v>
+      <c r="A12" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B13" s="3" t="s">
-        <v>17</v>
-      </c>
       <c r="C13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>18</v>
+      <c r="B14" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -816,33 +811,33 @@
         <v>10</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>10</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>26</v>
+        <v>10</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>27</v>
+      <c r="A16" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -850,119 +845,166 @@
         <v>18</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B18" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D18" s="2" t="s">
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="B27" s="6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="2" t="s">
+      <c r="C27" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D19" s="2" t="s">
+      <c r="D27" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="B28" s="6" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="B20" s="2" t="s">
+      <c r="C28" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D20" s="2" t="s">
+      <c r="D28" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="B29" s="6" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B21" s="2" t="s">
+      <c r="C29" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C23" s="2" t="s">
+      <c r="D29" s="6" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="2" t="s">
+      <c r="E29" s="6" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D30" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D31" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D32" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -973,7 +1015,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85833828-42CF-4E9A-8919-B3F15621B530}">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
@@ -1011,93 +1053,135 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="D3" s="2" t="s">
+      <c r="A3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="8" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="8" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D7" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C8" s="11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C9" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C10" s="10" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C8" s="7" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C11" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C9" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C10" s="4" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C11" s="2" t="s">
-        <v>18</v>
+      <c r="B13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -1124,12 +1208,12 @@
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="6" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="8" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1167,7 +1251,7 @@
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="7" t="s">
         <v>32</v>
       </c>
     </row>
@@ -1219,7 +1303,7 @@
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="8" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1265,7 +1349,7 @@
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="8" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1297,11 +1381,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="14" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
@@ -1315,13 +1399,13 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="12" t="s">
         <v>35</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1337,7 +1421,7 @@
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="6" t="s">
         <v>20</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1377,17 +1461,17 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
-        <v>42</v>
+      <c r="A1" s="5" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>41</v>
+      <c r="A2" s="13" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="7" t="s">
         <v>29</v>
       </c>
     </row>
@@ -1398,35 +1482,40 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ECFC2A7-8C30-4C6E-9B70-4D34865ED7BC}">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="7" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="7" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>43</v>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
20260322 Updated Table Link Processes
</commit_message>
<xml_diff>
--- a/reports.xlsx
+++ b/reports.xlsx
@@ -1,19 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IOtel\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{745FBCCF-4DCB-4880-A710-4DBE5CC06DE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1D34AA5-C871-4416-AAAC-9D61D8FFBF22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1080" windowWidth="17280" windowHeight="10500" xr2:uid="{4A38C952-6B38-47C9-B6BD-60FF9586BBD2}"/>
+    <workbookView xWindow="2928" yWindow="3900" windowWidth="17280" windowHeight="10500" firstSheet="4" activeTab="6" xr2:uid="{4A38C952-6B38-47C9-B6BD-60FF9586BBD2}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Reports" sheetId="1" r:id="rId1"/>
+    <sheet name="Schedules" sheetId="2" r:id="rId2"/>
+    <sheet name="Functions" sheetId="3" r:id="rId3"/>
+    <sheet name="Tags" sheetId="4" r:id="rId4"/>
+    <sheet name="Changes" sheetId="5" r:id="rId5"/>
+    <sheet name="SQL Statements" sheetId="6" r:id="rId6"/>
+    <sheet name="Tables" sheetId="7" r:id="rId7"/>
+    <sheet name="Publications" sheetId="8" r:id="rId8"/>
+    <sheet name="Linked Reports" sheetId="9" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,30 +43,162 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="8">
-  <si>
-    <t>begin</t>
-  </si>
-  <si>
-    <t>lees filter</t>
-  </si>
-  <si>
-    <t>filtype = leeg</t>
-  </si>
-  <si>
-    <t>filtype='reportType'</t>
-  </si>
-  <si>
-    <t>filtype = nie leeg</t>
-  </si>
-  <si>
-    <t>nie begin</t>
-  </si>
-  <si>
-    <t>fildet=filter.reportType</t>
-  </si>
-  <si>
-    <t>doen bywerking van filter tov filtype</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="52">
+  <si>
+    <t>Crystal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required </t>
+  </si>
+  <si>
+    <t>Report</t>
+  </si>
+  <si>
+    <t>Status</t>
+  </si>
+  <si>
+    <t>Source</t>
+  </si>
+  <si>
+    <t>Path</t>
+  </si>
+  <si>
+    <t>Components</t>
+  </si>
+  <si>
+    <t>Schedules</t>
+  </si>
+  <si>
+    <t>Functions</t>
+  </si>
+  <si>
+    <t>Tags</t>
+  </si>
+  <si>
+    <t>Changes</t>
+  </si>
+  <si>
+    <t>SQL statement</t>
+  </si>
+  <si>
+    <t>Tables</t>
+  </si>
+  <si>
+    <t>Add report</t>
+  </si>
+  <si>
+    <t>Edit Report</t>
+  </si>
+  <si>
+    <t>Remove Report</t>
+  </si>
+  <si>
+    <t>Select ion</t>
+  </si>
+  <si>
+    <t>Selection</t>
+  </si>
+  <si>
+    <t>Add</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add </t>
+  </si>
+  <si>
+    <t>View DB</t>
+  </si>
+  <si>
+    <t>Link Table</t>
+  </si>
+  <si>
+    <t>PHP</t>
+  </si>
+  <si>
+    <t>Recipients</t>
+  </si>
+  <si>
+    <t>Publications</t>
+  </si>
+  <si>
+    <t>Publication</t>
+  </si>
+  <si>
+    <t>Linked Reports</t>
+  </si>
+  <si>
+    <t>Filter</t>
+  </si>
+  <si>
+    <t>sh</t>
+  </si>
+  <si>
+    <t>View</t>
+  </si>
+  <si>
+    <t>Edit</t>
+  </si>
+  <si>
+    <t>Remove</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>Report selection</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>DB selection</t>
+  </si>
+  <si>
+    <t>Link Tables</t>
+  </si>
+  <si>
+    <t>DB Add</t>
+  </si>
+  <si>
+    <t>Link  Table</t>
+  </si>
+  <si>
+    <t>Table Selection</t>
+  </si>
+  <si>
+    <t>Crystal / PHP / Recipients</t>
+  </si>
+  <si>
+    <t>Crystal / Recipients</t>
+  </si>
+  <si>
+    <t>Show report Group</t>
+  </si>
+  <si>
+    <t>View Ricipients</t>
+  </si>
+  <si>
+    <t>View Report Schedule</t>
+  </si>
+  <si>
+    <t>View Publication  Schedule</t>
+  </si>
+  <si>
+    <t>Required</t>
+  </si>
+  <si>
+    <t>runTime</t>
+  </si>
+  <si>
+    <t>Dest Detail</t>
+  </si>
+  <si>
+    <t>Local</t>
+  </si>
+  <si>
+    <t>Custom</t>
+  </si>
+  <si>
+    <t>Update Done</t>
   </si>
 </sst>
 </file>
@@ -74,12 +214,24 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -94,10 +246,47 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="4"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="5"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -418,56 +607,949 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92C6B047-5BD0-4FE0-9344-E232D0E4E58E}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr defaultColWidth="12.33203125" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C16" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E16" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="C23" s="8" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C26" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B29" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D30" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D31" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D32" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E32" s="8" t="s">
+        <v>17</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85833828-42CF-4E9A-8919-B3F15621B530}">
+  <dimension ref="A1:D15"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C8" s="11" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C9" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C10" s="10" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="C11" s="6" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" t="s">
+        <v>46</v>
+      </c>
+      <c r="C13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0EFCA283-128B-472C-881B-44B4853A4854}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B3" s="1" t="s">
-        <v>3</v>
+      <c r="A3" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B4" s="1" t="s">
-        <v>6</v>
+      <c r="A4" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>5</v>
+      <c r="A5" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="8" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1</v>
+      <c r="A6" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>31</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B7" t="s">
-        <v>7</v>
+      <c r="A7" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{485339A9-4BE2-45AB-8FCB-653A83302CB3}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="7" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="3"/>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="3"/>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D83B7FB6-87DE-4BE7-B4DF-F791D9A03C62}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8204F7E-C86F-4DDB-AB30-05192EA3866B}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{789D6D66-3E83-4E10-B02B-B18567320797}">
+  <dimension ref="A1:C7"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="2" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="8" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F93FCF0B-DF71-4561-B3D8-C995E16F98A3}">
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="13" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ECFC2A7-8C30-4C6E-9B70-4D34865ED7BC}">
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="12" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
2026-3-27 Made more Link Table updates
</commit_message>
<xml_diff>
--- a/reports.xlsx
+++ b/reports.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IOtel\Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1D34AA5-C871-4416-AAAC-9D61D8FFBF22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFEF14CE-B88A-4AF4-804B-FF5D804ABD61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2928" yWindow="3900" windowWidth="17280" windowHeight="10500" firstSheet="4" activeTab="6" xr2:uid="{4A38C952-6B38-47C9-B6BD-60FF9586BBD2}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="10" xr2:uid="{4A38C952-6B38-47C9-B6BD-60FF9586BBD2}"/>
   </bookViews>
   <sheets>
     <sheet name="Reports" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,8 @@
     <sheet name="Tables" sheetId="7" r:id="rId7"/>
     <sheet name="Publications" sheetId="8" r:id="rId8"/>
     <sheet name="Linked Reports" sheetId="9" r:id="rId9"/>
+    <sheet name="Var Names" sheetId="10" r:id="rId10"/>
+    <sheet name="Lists" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="212" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="63">
   <si>
     <t>Crystal</t>
   </si>
@@ -199,6 +201,39 @@
   </si>
   <si>
     <t>Update Done</t>
+  </si>
+  <si>
+    <t>lstRepType</t>
+  </si>
+  <si>
+    <t>lstPath</t>
+  </si>
+  <si>
+    <t>lstStatus</t>
+  </si>
+  <si>
+    <t>lstDB</t>
+  </si>
+  <si>
+    <t>lstdbType</t>
+  </si>
+  <si>
+    <t>lstServer</t>
+  </si>
+  <si>
+    <t>lstFormat</t>
+  </si>
+  <si>
+    <t>lstTabInput</t>
+  </si>
+  <si>
+    <t>lstRecurrence</t>
+  </si>
+  <si>
+    <t>lstSource</t>
+  </si>
+  <si>
+    <t>lstTag</t>
   </si>
 </sst>
 </file>
@@ -308,6 +343,693 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>381667</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>95478</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D9B48E96-EBB4-BA49-3BD2-520F35526D44}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7696867" cy="2629128"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>15240</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>207645</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>80007</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="20" name="Group 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{25C690CF-3861-2FDC-EC4E-35515EDB97D3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="281940" y="200025"/>
+          <a:ext cx="4196715" cy="2956557"/>
+          <a:chOff x="285750" y="196215"/>
+          <a:chExt cx="4189095" cy="2960367"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="9" name="Straight Arrow Connector 8">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{63ADF1E9-9674-4F6B-82DF-6E4C012A0847}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm flipH="1" flipV="1">
+            <a:off x="285750" y="1360170"/>
+            <a:ext cx="393751" cy="1649730"/>
+          </a:xfrm>
+          <a:prstGeom prst="straightConnector1">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="7" name="TextBox 6">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8FC89C64-B6DD-5425-19C8-2C53194BAB06}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="612090" y="2913745"/>
+            <a:ext cx="552041" cy="242837"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="lt1"/>
+          </a:solidFill>
+          <a:ln w="9525" cmpd="sng">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:rPr lang="en-ZA" sz="1100"/>
+              <a:t>selrep</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="10" name="Straight Arrow Connector 9">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{431A83E0-1E69-4350-B21D-52938EBF8702}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm flipH="1" flipV="1">
+            <a:off x="359907" y="198111"/>
+            <a:ext cx="528046" cy="2712884"/>
+          </a:xfrm>
+          <a:prstGeom prst="straightConnector1">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="12" name="Straight Arrow Connector 11">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F23BF802-6CB5-4FCF-B109-45C54ADDB3CC}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr>
+            <a:stCxn id="7" idx="3"/>
+          </xdr:cNvCxnSpPr>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm flipV="1">
+            <a:off x="1160321" y="196215"/>
+            <a:ext cx="3314524" cy="2835139"/>
+          </a:xfrm>
+          <a:prstGeom prst="straightConnector1">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>592455</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>129540</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>76200</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>24765</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="21" name="Group 20">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B2B251F2-7B69-EB10-FBB9-61AB709C59ED}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="4855845" y="2486025"/>
+          <a:ext cx="706755" cy="611505"/>
+          <a:chOff x="4859655" y="2482215"/>
+          <a:chExt cx="702945" cy="619125"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="14" name="TextBox 13">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8B248141-9A36-C0CF-6FE7-C8B58D3976BA}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="4859655" y="2849880"/>
+            <a:ext cx="702945" cy="251460"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="lt1"/>
+          </a:solidFill>
+          <a:ln w="9525" cmpd="sng">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:rPr lang="en-ZA" sz="1100"/>
+              <a:t>selcomp</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:endParaRPr lang="en-ZA" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="15" name="Straight Arrow Connector 14">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54262237-A4A4-45D2-9B35-336E615D640E}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm flipV="1">
+            <a:off x="5145405" y="2482215"/>
+            <a:ext cx="177165" cy="361950"/>
+          </a:xfrm>
+          <a:prstGeom prst="straightConnector1">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>167640</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>93345</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>36910</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="26" name="Group 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{39B20734-CD18-192E-8785-369D0556BCEA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="6096000" y="2524125"/>
+          <a:ext cx="706755" cy="589360"/>
+          <a:chOff x="6096000" y="2520315"/>
+          <a:chExt cx="702945" cy="593170"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="24" name="TextBox 23">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{13F20A5C-A87C-4CC0-8768-10B70D3E6656}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6096000" y="2867025"/>
+            <a:ext cx="702945" cy="246460"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="lt1"/>
+          </a:solidFill>
+          <a:ln w="9525" cmpd="sng">
+            <a:solidFill>
+              <a:schemeClr val="lt1">
+                <a:shade val="50000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="dk1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:rPr lang="en-ZA" sz="1100"/>
+              <a:t>cmpsel</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:endParaRPr lang="en-ZA" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:cxnSp macro="">
+        <xdr:nvCxnSpPr>
+          <xdr:cNvPr id="25" name="Straight Arrow Connector 24">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4552A0CE-3ED9-4AA0-A565-6A6CEED7B839}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvCxnSpPr/>
+        </xdr:nvCxnSpPr>
+        <xdr:spPr>
+          <a:xfrm flipV="1">
+            <a:off x="6515100" y="2520315"/>
+            <a:ext cx="174315" cy="365115"/>
+          </a:xfrm>
+          <a:prstGeom prst="straightConnector1">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:tailEnd type="triangle"/>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+      </xdr:cxnSp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>19</xdr:col>
+      <xdr:colOff>590865</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>121970</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="27" name="Picture 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7745763D-6FB4-D66F-BDFF-0CBED467F302}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="8534400" y="95250"/>
+          <a:ext cx="3638865" cy="569645"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>605791</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>5715</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>590551</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>60092</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="30" name="TextBox 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72E00D72-CC14-4620-A53F-AB9552DA1983}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10359391" y="910590"/>
+          <a:ext cx="594360" cy="235352"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-ZA" sz="1100"/>
+            <a:t>selact</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="en-ZA" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>352425</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>520065</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>38920</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="31" name="Straight Arrow Connector 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{763FFD23-CB66-4BA8-883C-780EB292AABF}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipV="1">
+          <a:off x="10715625" y="581025"/>
+          <a:ext cx="167640" cy="362770"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:tailEnd type="triangle"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1022,6 +1744,84 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A558CBCD-630A-4295-8B5E-B4193C094478}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C825EF94-6465-4B50-95EF-7789B743101D}">
+  <dimension ref="A2:A12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="12.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>62</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85833828-42CF-4E9A-8919-B3F15621B530}">
   <dimension ref="A1:D15"/>

</xml_diff>